<commit_message>
Update test cases Excel file
</commit_message>
<xml_diff>
--- a/IT23150034_Test_Cases.xlsx
+++ b/IT23150034_Test_Cases.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PCSM\Desktop\IT23150034\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{16AC509B-8FE2-4995-BD05-9D04CDB83327}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C9D6B29E-3304-4203-A599-6B4DA08A26C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="257" uniqueCount="183">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="357" uniqueCount="233">
   <si>
     <t>TC ID</t>
   </si>
@@ -58,6 +58,12 @@
     <t>මම යන්න ඕනි</t>
   </si>
   <si>
+    <t>මම යන ඕනි</t>
+  </si>
+  <si>
+    <t>FAIL</t>
+  </si>
+  <si>
     <t>Neg_02</t>
   </si>
   <si>
@@ -70,6 +76,9 @@
     <t>මම හිතනවා අපි හෙට උදේ කන්න ඕනි කියලා</t>
   </si>
   <si>
+    <t>මම හිතනවා අපි හෙට උදේට කන්න ඕනි කියලා</t>
+  </si>
+  <si>
     <t>Neg_03</t>
   </si>
   <si>
@@ -82,6 +91,9 @@
     <t>හොඳ නේද</t>
   </si>
   <si>
+    <t>හොද නේද</t>
+  </si>
+  <si>
     <t>Neg_04</t>
   </si>
   <si>
@@ -91,6 +103,9 @@
     <t>ඔයා හොඳ නේද කියලා මම අහන්නේ දැනගන්න</t>
   </si>
   <si>
+    <t>ඔයා හොද නේද කියලා මම අහන්නේ දැනගන්න</t>
+  </si>
+  <si>
     <t>Neg_05</t>
   </si>
   <si>
@@ -103,6 +118,9 @@
     <t>මට කනවා</t>
   </si>
   <si>
+    <t>මාත් කනවා</t>
+  </si>
+  <si>
     <t>Neg_06</t>
   </si>
   <si>
@@ -112,6 +130,9 @@
     <t>මට කනවා කියලා මම කිව්වා නිසා ඔයාට තේරුනා නෑ</t>
   </si>
   <si>
+    <t>මමත් කනවා කියලා මම කිව්වා නිසා ඔයාට තේරුනා නෑ</t>
+  </si>
+  <si>
     <t>Neg_07</t>
   </si>
   <si>
@@ -124,6 +145,9 @@
     <t>මාර කෑමක් උනා</t>
   </si>
   <si>
+    <t>මාරු කෑමක් උනා</t>
+  </si>
+  <si>
     <t>Neg_08</t>
   </si>
   <si>
@@ -133,6 +157,9 @@
     <t>අද මාර කෑමක් උනා කියලා මම සෙට් එකට කිව්වා</t>
   </si>
   <si>
+    <t>අද මාරු කෑමක් උනා කියලා මම set එකට කිව්වා</t>
+  </si>
+  <si>
     <t>Neg_09</t>
   </si>
   <si>
@@ -145,6 +172,9 @@
     <t>මම බස් එකට ගියා</t>
   </si>
   <si>
+    <t>මම bus එකට ගියා</t>
+  </si>
+  <si>
     <t>Neg_10</t>
   </si>
   <si>
@@ -154,6 +184,9 @@
     <t>මම බස් එකට ගියා කියලා මම ඔයාට කියන්න හිත ගියා</t>
   </si>
   <si>
+    <t>මම bus එකට ගියා කියලා මම ඔයාට කියන්න හිතා ගියා</t>
+  </si>
+  <si>
     <t>Neg_11</t>
   </si>
   <si>
@@ -166,6 +199,9 @@
     <t>ඔයා ඉක්මනට එනවා</t>
   </si>
   <si>
+    <t>ඔයා brb</t>
+  </si>
+  <si>
     <t>Neg_12</t>
   </si>
   <si>
@@ -175,6 +211,9 @@
     <t>ඔයා ඉක්මනට එනවා කියලා මම කිව්වා නිසා ඔයාට අව්ලක් නෑ</t>
   </si>
   <si>
+    <t>ඔයා brb කියලා මම කිව්වා නිසා ඔයාට අව්ලක් නෑ</t>
+  </si>
+  <si>
     <t>Neg_13</t>
   </si>
   <si>
@@ -187,6 +226,9 @@
     <t>මම අද එනවා</t>
   </si>
   <si>
+    <t>මම 2දේ එනවා</t>
+  </si>
+  <si>
     <t>Neg_14</t>
   </si>
   <si>
@@ -196,6 +238,9 @@
     <t>මම අද එනවා කියලා මම කිව්වා නිසා ඔයාට දැනගන්න පුළුවන්</t>
   </si>
   <si>
+    <t>මම 2දේ එනවා කියලා මම කිව්වා නිසා ඔයාට දෑනගන්න පුළුවන්</t>
+  </si>
+  <si>
     <t>Neg_15</t>
   </si>
   <si>
@@ -208,6 +253,9 @@
     <t>එයා නේ</t>
   </si>
   <si>
+    <t>එයානේ</t>
+  </si>
+  <si>
     <t>Neg_16</t>
   </si>
   <si>
@@ -217,6 +265,9 @@
     <t>මම හිතන්නේ එක හරි ඔව් කියලා ඔයාට කියන්න</t>
   </si>
   <si>
+    <t>මම හිතන්නේ ඒක හරි ඇයි කියලා ඔයාට කියන්න</t>
+  </si>
+  <si>
     <t>Neg_17</t>
   </si>
   <si>
@@ -238,6 +289,9 @@
     <t>ඔයා යනවා කියලා මම හිතනවා එහෙම නෙමෙයි කියලා</t>
   </si>
   <si>
+    <t>oyayanawa කියලා මම හිතනවා එහෙම නෙමේ කියලා</t>
+  </si>
+  <si>
     <t>Neg_19</t>
   </si>
   <si>
@@ -250,6 +304,9 @@
     <t>මම කනවා</t>
   </si>
   <si>
+    <t>මම කන්නවා</t>
+  </si>
+  <si>
     <t>Neg_20</t>
   </si>
   <si>
@@ -259,6 +316,9 @@
     <t>මම කනවා කියලා මම capital use කළා නිසා වැරදි උනා</t>
   </si>
   <si>
+    <t>මම කනවා කියලා මම Capital use කළා නිසා වැරදි වුණා</t>
+  </si>
+  <si>
     <t>Neg_21</t>
   </si>
   <si>
@@ -271,6 +331,9 @@
     <t>ඔයා ආවද</t>
   </si>
   <si>
+    <t>ඔයා ආව ද!!!</t>
+  </si>
+  <si>
     <t>Neg_22</t>
   </si>
   <si>
@@ -280,6 +343,9 @@
     <t>ඔයා ආවද කියලා මම ඇහුවට එයා හරියට හදන්න බැහැ</t>
   </si>
   <si>
+    <t>ඔයා ආව ද!!! කියලා මම අහුවට එයා හරියට හදන්න බෑ</t>
+  </si>
+  <si>
     <t>Neg_23</t>
   </si>
   <si>
@@ -292,6 +358,9 @@
     <t>වාව්</t>
   </si>
   <si>
+    <t>වොඔව්</t>
+  </si>
+  <si>
     <t>Neg_24</t>
   </si>
   <si>
@@ -301,6 +370,9 @@
     <t>වාව් කියලා මම කියන්නේ එයා එහෙම කරන්න එපා කියලා</t>
   </si>
   <si>
+    <t>වොඔව් කියලා මම කියන්නේ එයා එහෙම කරන්න එපා කියලා</t>
+  </si>
+  <si>
     <t>Neg_25</t>
   </si>
   <si>
@@ -313,6 +385,9 @@
     <t>උඹ එනවා</t>
   </si>
   <si>
+    <t>උඹ එන්නව</t>
+  </si>
+  <si>
     <t>Neg_26</t>
   </si>
   <si>
@@ -322,6 +397,9 @@
     <t>උඹ එනවා කියලා මම කිව්වා නිසා එයා තේරුම් ගත්ත</t>
   </si>
   <si>
+    <t>උඹ එනවා කියලා මම කිව්වා නිසා එයා තේරුම් ගත්තා</t>
+  </si>
+  <si>
     <t>Neg_27</t>
   </si>
   <si>
@@ -334,6 +412,9 @@
     <t>අපි ආවා</t>
   </si>
   <si>
+    <t>ආවා අපි</t>
+  </si>
+  <si>
     <t>Neg_28</t>
   </si>
   <si>
@@ -343,6 +424,9 @@
     <t>අපි ආවා කියලා මම කිව්වා නිසා එකට වෙනසක් තියෙනවා</t>
   </si>
   <si>
+    <t>ආවා අපි කියලා මම කිව්වා නිසා ඒකට වෙනසක් තියෙනවා</t>
+  </si>
+  <si>
     <t>Neg_29</t>
   </si>
   <si>
@@ -355,6 +439,9 @@
     <t>මම යනවා</t>
   </si>
   <si>
+    <t>මම් යනවා</t>
+  </si>
+  <si>
     <t>Neg_30</t>
   </si>
   <si>
@@ -364,6 +451,9 @@
     <t>මම යනවා කියලා මම type කරද්දී පොඩි වැරද්දක් උනා</t>
   </si>
   <si>
+    <t>මම් යනවා කියලා මම type කරද්දි පොඩි වරද්දක් උනා</t>
+  </si>
+  <si>
     <t>Neg_31</t>
   </si>
   <si>
@@ -376,6 +466,9 @@
     <t>කරුද</t>
   </si>
   <si>
+    <t>කාරුවද</t>
+  </si>
+  <si>
     <t>Neg_32</t>
   </si>
   <si>
@@ -385,6 +478,9 @@
     <t>එයා කරු වැඩ කරනවා කියලා මම හිතනවා</t>
   </si>
   <si>
+    <t>එයා කරු වැඩ කරනවා කියලා මම හිතන්නවා</t>
+  </si>
+  <si>
     <t>Neg_33</t>
   </si>
   <si>
@@ -397,6 +493,9 @@
     <t>මටනම් බැහැ</t>
   </si>
   <si>
+    <t>මටන්නම් බැහැ</t>
+  </si>
+  <si>
     <t>Neg_34</t>
   </si>
   <si>
@@ -406,6 +505,9 @@
     <t>බැහැ කියලා මම කිව්වා නිසා ඔයාට එක තේරුනා</t>
   </si>
   <si>
+    <t>බැහැ කියලා මම කිව්වා නිසා ඔයාට ඒක තේරුණා</t>
+  </si>
+  <si>
     <t>Neg_35</t>
   </si>
   <si>
@@ -418,6 +520,9 @@
     <t>ඔයා අහනවද මේක</t>
   </si>
   <si>
+    <t>ඔයා අහනවද මේකේ</t>
+  </si>
+  <si>
     <t>Neg_36</t>
   </si>
   <si>
@@ -427,6 +532,9 @@
     <t>ඔයා අහනවද මේක කරන්න කියලා මම අහන්නේ</t>
   </si>
   <si>
+    <t>ඔයා අහනවද මේක කරන්න කියල මම අහන්නෙ</t>
+  </si>
+  <si>
     <t>Neg_37</t>
   </si>
   <si>
@@ -439,6 +547,9 @@
     <t>මම කමින් ඉන්නවා</t>
   </si>
   <si>
+    <t>මම කනවා ඉන්නේ</t>
+  </si>
+  <si>
     <t>Neg_38</t>
   </si>
   <si>
@@ -448,6 +559,9 @@
     <t>මම කමින් ඉන්නවා කියලා මම කිව්වා නිසා එකට වෙනසක් තියෙනවා</t>
   </si>
   <si>
+    <t>මම කනවා ඉන්නේ කියලා මම කිව්වා නිසා ඒකට වෙනසක් තියෙනවා</t>
+  </si>
+  <si>
     <t>Neg_39</t>
   </si>
   <si>
@@ -460,6 +574,9 @@
     <t>අපි ගියා</t>
   </si>
   <si>
+    <t>අපිගියා</t>
+  </si>
+  <si>
     <t>Neg_40</t>
   </si>
   <si>
@@ -469,6 +586,9 @@
     <t>අපි ගියා කියලා මම කිව්වා නිසා ඔයාට තේරුනා නෑ</t>
   </si>
   <si>
+    <t>අපි ගියා කියලා මම කිව නිසා ඔයාට තේරුනේ නෑ</t>
+  </si>
+  <si>
     <t>Neg_41</t>
   </si>
   <si>
@@ -481,6 +601,9 @@
     <t>එක ගන්න</t>
   </si>
   <si>
+    <t>ඒක ගන</t>
+  </si>
+  <si>
     <t>Neg_42</t>
   </si>
   <si>
@@ -490,6 +613,9 @@
     <t>එක ගන්න කියලා මම කිව්වා නිසා එයා ගන්න ඕනි</t>
   </si>
   <si>
+    <t>ඒක ගන්න කියලා මම කිව්වා නිසා එයා ගන්න ඕනි</t>
+  </si>
+  <si>
     <t>Neg_43</t>
   </si>
   <si>
@@ -502,6 +628,9 @@
     <t>බෑග් එක දෙන්න</t>
   </si>
   <si>
+    <t>bag එක දෙන්න</t>
+  </si>
+  <si>
     <t>Neg_44</t>
   </si>
   <si>
@@ -511,6 +640,9 @@
     <t>බෑග් එක දෙන්න කියලා මම කිව්වා නිසා එයා එක දෙන්න පුළුවන්</t>
   </si>
   <si>
+    <t>bag එක දෙන්න කියලා මම කිව්වා නිසා එයා එක දෙන්න පුළුවන්</t>
+  </si>
+  <si>
     <t>Neg_45</t>
   </si>
   <si>
@@ -523,6 +655,9 @@
     <t>යන්න ඕනි</t>
   </si>
   <si>
+    <t>යන්නඕනි</t>
+  </si>
+  <si>
     <t>Neg_46</t>
   </si>
   <si>
@@ -532,6 +667,9 @@
     <t>යන්න ඕනි කියලා මම කිව්වා නිසා අපි මේක කරමු</t>
   </si>
   <si>
+    <t>යන්න ඕනි කියලා මම කිව නිසා අපි මේක කරමු</t>
+  </si>
+  <si>
     <t>Neg_47</t>
   </si>
   <si>
@@ -541,6 +679,9 @@
     <t>mama eat karanawa</t>
   </si>
   <si>
+    <t>මම eat කරනවා</t>
+  </si>
+  <si>
     <t>Neg_48</t>
   </si>
   <si>
@@ -550,6 +691,9 @@
     <t>මම කනවා කියලා මම කිව්වා නිසා එක හරියට වෙනස් උනා</t>
   </si>
   <si>
+    <t>මම eat කරනවා කියලා මම කිව්වා නිසා ඒක හරියට වෙනස් උනා</t>
+  </si>
+  <si>
     <t>Neg_49</t>
   </si>
   <si>
@@ -562,6 +706,9 @@
     <t>කොහෙද ඔයාගේ කාර්යාලය</t>
   </si>
   <si>
+    <t>කොහෙද ඔයාගෙ office</t>
+  </si>
+  <si>
     <t>Neg_50</t>
   </si>
   <si>
@@ -569,6 +716,9 @@
   </si>
   <si>
     <t>කොහෙද ඔයාගේ කාර්යාලය කියලා මම අහන්නේ ඔයාට හොඳද කියලා</t>
+  </si>
+  <si>
+    <t>කොහෙද ඔයාගේ office කියලා මම අහන්නේ ඔයාට හොඳ ද කියලා</t>
   </si>
 </sst>
 </file>
@@ -647,7 +797,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -658,10 +808,16 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1021,939 +1177,1139 @@
       <c r="E2" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="F2" s="3"/>
-      <c r="G2" s="4"/>
+      <c r="F2" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="G2" s="7" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="3" spans="1:7" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A3" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="B3" s="5" t="s">
+      <c r="A3" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="B3" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="C3" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="D3" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="E3" s="6" t="s">
+      <c r="C3" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="F3" s="6"/>
-      <c r="G3" s="7"/>
+      <c r="D3" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="F3" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="G3" s="9" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>9</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="F4" s="3"/>
-      <c r="G4" s="4"/>
+        <v>22</v>
+      </c>
+      <c r="F4" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="G4" s="7" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="5" spans="1:7" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A5" s="5" t="s">
+      <c r="A5" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="B5" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="B5" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="C5" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="D5" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="E5" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="F5" s="6"/>
-      <c r="G5" s="7"/>
+      <c r="C5" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="F5" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="G5" s="9" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>9</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="F6" s="3"/>
-      <c r="G6" s="4"/>
+        <v>31</v>
+      </c>
+      <c r="F6" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="G6" s="7" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="7" spans="1:7" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A7" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="B7" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="C7" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="D7" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="E7" s="6" t="s">
+      <c r="A7" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="B7" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="F7" s="6"/>
-      <c r="G7" s="7"/>
+      <c r="C7" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="E7" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="F7" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="G7" s="9" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
-        <v>30</v>
+        <v>37</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>31</v>
+        <v>38</v>
       </c>
       <c r="C8" s="2" t="s">
         <v>9</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>32</v>
+        <v>39</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="F8" s="3"/>
-      <c r="G8" s="4"/>
+        <v>40</v>
+      </c>
+      <c r="F8" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="G8" s="7" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="9" spans="1:7" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A9" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="B9" s="5" t="s">
-        <v>31</v>
-      </c>
-      <c r="C9" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="D9" s="6" t="s">
-        <v>35</v>
-      </c>
-      <c r="E9" s="6" t="s">
-        <v>36</v>
-      </c>
-      <c r="F9" s="6"/>
-      <c r="G9" s="7"/>
+      <c r="A9" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="D9" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="E9" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="F9" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="G9" s="9" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
-        <v>37</v>
+        <v>46</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>38</v>
+        <v>47</v>
       </c>
       <c r="C10" s="2" t="s">
         <v>9</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>39</v>
+        <v>48</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="F10" s="3"/>
-      <c r="G10" s="4"/>
+        <v>49</v>
+      </c>
+      <c r="F10" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="G10" s="7" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="11" spans="1:7" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A11" s="5" t="s">
-        <v>41</v>
-      </c>
-      <c r="B11" s="5" t="s">
-        <v>38</v>
-      </c>
-      <c r="C11" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="D11" s="6" t="s">
-        <v>42</v>
-      </c>
-      <c r="E11" s="6" t="s">
-        <v>43</v>
-      </c>
-      <c r="F11" s="6"/>
-      <c r="G11" s="7"/>
+      <c r="A11" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="D11" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="E11" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="F11" s="8" t="s">
+        <v>54</v>
+      </c>
+      <c r="G11" s="9" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
-        <v>44</v>
+        <v>55</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>45</v>
+        <v>56</v>
       </c>
       <c r="C12" s="2" t="s">
         <v>9</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>46</v>
+        <v>57</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="F12" s="3"/>
-      <c r="G12" s="4"/>
+        <v>58</v>
+      </c>
+      <c r="F12" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="G12" s="7" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="13" spans="1:7" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A13" s="5" t="s">
-        <v>48</v>
-      </c>
-      <c r="B13" s="5" t="s">
-        <v>45</v>
-      </c>
-      <c r="C13" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="D13" s="6" t="s">
-        <v>49</v>
-      </c>
-      <c r="E13" s="6" t="s">
-        <v>50</v>
-      </c>
-      <c r="F13" s="6"/>
-      <c r="G13" s="7"/>
+      <c r="A13" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D13" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="E13" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="F13" s="8" t="s">
+        <v>63</v>
+      </c>
+      <c r="G13" s="9" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
-        <v>51</v>
+        <v>64</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>52</v>
+        <v>65</v>
       </c>
       <c r="C14" s="2" t="s">
         <v>9</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>53</v>
+        <v>66</v>
       </c>
       <c r="E14" s="3" t="s">
-        <v>54</v>
-      </c>
-      <c r="F14" s="3"/>
-      <c r="G14" s="4"/>
+        <v>67</v>
+      </c>
+      <c r="F14" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="G14" s="7" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="15" spans="1:7" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A15" s="5" t="s">
-        <v>55</v>
-      </c>
-      <c r="B15" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="C15" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="D15" s="6" t="s">
-        <v>56</v>
-      </c>
-      <c r="E15" s="6" t="s">
-        <v>57</v>
-      </c>
-      <c r="F15" s="6"/>
-      <c r="G15" s="7"/>
+      <c r="A15" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="D15" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="E15" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="F15" s="8" t="s">
+        <v>72</v>
+      </c>
+      <c r="G15" s="9" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A16" s="2" t="s">
-        <v>58</v>
+        <v>73</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>59</v>
+        <v>74</v>
       </c>
       <c r="C16" s="2" t="s">
         <v>9</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>60</v>
+        <v>75</v>
       </c>
       <c r="E16" s="3" t="s">
-        <v>61</v>
-      </c>
-      <c r="F16" s="3"/>
-      <c r="G16" s="4"/>
+        <v>76</v>
+      </c>
+      <c r="F16" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="G16" s="7" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="17" spans="1:7" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A17" s="5" t="s">
-        <v>62</v>
-      </c>
-      <c r="B17" s="5" t="s">
-        <v>59</v>
-      </c>
-      <c r="C17" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="D17" s="6" t="s">
-        <v>63</v>
-      </c>
-      <c r="E17" s="6" t="s">
-        <v>64</v>
-      </c>
-      <c r="F17" s="6"/>
-      <c r="G17" s="7"/>
+      <c r="A17" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="B17" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="C17" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="D17" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="E17" s="5" t="s">
+        <v>80</v>
+      </c>
+      <c r="F17" s="8" t="s">
+        <v>81</v>
+      </c>
+      <c r="G17" s="9" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A18" s="2" t="s">
-        <v>65</v>
+        <v>82</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>66</v>
+        <v>83</v>
       </c>
       <c r="C18" s="2" t="s">
         <v>9</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>67</v>
+        <v>84</v>
       </c>
       <c r="E18" s="3" t="s">
-        <v>68</v>
-      </c>
-      <c r="F18" s="3"/>
-      <c r="G18" s="4"/>
+        <v>85</v>
+      </c>
+      <c r="F18" s="6" t="s">
+        <v>84</v>
+      </c>
+      <c r="G18" s="7" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="19" spans="1:7" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A19" s="5" t="s">
-        <v>69</v>
-      </c>
-      <c r="B19" s="5" t="s">
-        <v>66</v>
-      </c>
-      <c r="C19" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="D19" s="6" t="s">
-        <v>70</v>
-      </c>
-      <c r="E19" s="6" t="s">
-        <v>71</v>
-      </c>
-      <c r="F19" s="6"/>
-      <c r="G19" s="7"/>
+      <c r="A19" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="B19" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="C19" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="D19" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="E19" s="5" t="s">
+        <v>88</v>
+      </c>
+      <c r="F19" s="8" t="s">
+        <v>89</v>
+      </c>
+      <c r="G19" s="9" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A20" s="2" t="s">
-        <v>72</v>
+        <v>90</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>73</v>
+        <v>91</v>
       </c>
       <c r="C20" s="2" t="s">
         <v>9</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>74</v>
+        <v>92</v>
       </c>
       <c r="E20" s="3" t="s">
-        <v>75</v>
-      </c>
-      <c r="F20" s="3"/>
-      <c r="G20" s="4"/>
+        <v>93</v>
+      </c>
+      <c r="F20" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="G20" s="7" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="21" spans="1:7" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A21" s="5" t="s">
-        <v>76</v>
-      </c>
-      <c r="B21" s="5" t="s">
-        <v>73</v>
-      </c>
-      <c r="C21" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="D21" s="6" t="s">
-        <v>77</v>
-      </c>
-      <c r="E21" s="6" t="s">
-        <v>78</v>
-      </c>
-      <c r="F21" s="6"/>
-      <c r="G21" s="7"/>
+      <c r="A21" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="B21" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="C21" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="D21" s="5" t="s">
+        <v>96</v>
+      </c>
+      <c r="E21" s="5" t="s">
+        <v>97</v>
+      </c>
+      <c r="F21" s="8" t="s">
+        <v>98</v>
+      </c>
+      <c r="G21" s="9" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A22" s="2" t="s">
-        <v>79</v>
+        <v>99</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="C22" s="2" t="s">
         <v>9</v>
       </c>
       <c r="D22" s="3" t="s">
-        <v>81</v>
+        <v>101</v>
       </c>
       <c r="E22" s="3" t="s">
-        <v>82</v>
-      </c>
-      <c r="F22" s="3"/>
-      <c r="G22" s="4"/>
+        <v>102</v>
+      </c>
+      <c r="F22" s="6" t="s">
+        <v>103</v>
+      </c>
+      <c r="G22" s="7" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="23" spans="1:7" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A23" s="5" t="s">
-        <v>83</v>
-      </c>
-      <c r="B23" s="5" t="s">
-        <v>80</v>
-      </c>
-      <c r="C23" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="D23" s="6" t="s">
-        <v>84</v>
-      </c>
-      <c r="E23" s="6" t="s">
-        <v>85</v>
-      </c>
-      <c r="F23" s="6"/>
-      <c r="G23" s="7"/>
+      <c r="A23" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="B23" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="C23" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="D23" s="5" t="s">
+        <v>105</v>
+      </c>
+      <c r="E23" s="5" t="s">
+        <v>106</v>
+      </c>
+      <c r="F23" s="8" t="s">
+        <v>107</v>
+      </c>
+      <c r="G23" s="9" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A24" s="2" t="s">
-        <v>86</v>
+        <v>108</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>87</v>
+        <v>109</v>
       </c>
       <c r="C24" s="2" t="s">
         <v>9</v>
       </c>
       <c r="D24" s="3" t="s">
-        <v>88</v>
+        <v>110</v>
       </c>
       <c r="E24" s="3" t="s">
-        <v>89</v>
-      </c>
-      <c r="F24" s="3"/>
-      <c r="G24" s="4"/>
+        <v>111</v>
+      </c>
+      <c r="F24" s="6" t="s">
+        <v>112</v>
+      </c>
+      <c r="G24" s="7" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="25" spans="1:7" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A25" s="5" t="s">
-        <v>90</v>
-      </c>
-      <c r="B25" s="5" t="s">
-        <v>87</v>
-      </c>
-      <c r="C25" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="D25" s="6" t="s">
-        <v>91</v>
-      </c>
-      <c r="E25" s="6" t="s">
-        <v>92</v>
-      </c>
-      <c r="F25" s="6"/>
-      <c r="G25" s="7"/>
+      <c r="A25" s="4" t="s">
+        <v>113</v>
+      </c>
+      <c r="B25" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="C25" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="D25" s="5" t="s">
+        <v>114</v>
+      </c>
+      <c r="E25" s="5" t="s">
+        <v>115</v>
+      </c>
+      <c r="F25" s="8" t="s">
+        <v>116</v>
+      </c>
+      <c r="G25" s="9" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A26" s="2" t="s">
-        <v>93</v>
+        <v>117</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>94</v>
+        <v>118</v>
       </c>
       <c r="C26" s="2" t="s">
         <v>9</v>
       </c>
       <c r="D26" s="3" t="s">
-        <v>95</v>
+        <v>119</v>
       </c>
       <c r="E26" s="3" t="s">
-        <v>96</v>
-      </c>
-      <c r="F26" s="3"/>
-      <c r="G26" s="4"/>
+        <v>120</v>
+      </c>
+      <c r="F26" s="6" t="s">
+        <v>121</v>
+      </c>
+      <c r="G26" s="7" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="27" spans="1:7" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A27" s="5" t="s">
-        <v>97</v>
-      </c>
-      <c r="B27" s="5" t="s">
-        <v>94</v>
-      </c>
-      <c r="C27" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="D27" s="6" t="s">
-        <v>98</v>
-      </c>
-      <c r="E27" s="6" t="s">
-        <v>99</v>
-      </c>
-      <c r="F27" s="6"/>
-      <c r="G27" s="7"/>
+      <c r="A27" s="4" t="s">
+        <v>122</v>
+      </c>
+      <c r="B27" s="4" t="s">
+        <v>118</v>
+      </c>
+      <c r="C27" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="D27" s="5" t="s">
+        <v>123</v>
+      </c>
+      <c r="E27" s="5" t="s">
+        <v>124</v>
+      </c>
+      <c r="F27" s="8" t="s">
+        <v>125</v>
+      </c>
+      <c r="G27" s="9" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A28" s="2" t="s">
-        <v>100</v>
+        <v>126</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>101</v>
+        <v>127</v>
       </c>
       <c r="C28" s="2" t="s">
         <v>9</v>
       </c>
       <c r="D28" s="3" t="s">
-        <v>102</v>
+        <v>128</v>
       </c>
       <c r="E28" s="3" t="s">
-        <v>103</v>
-      </c>
-      <c r="F28" s="3"/>
-      <c r="G28" s="4"/>
+        <v>129</v>
+      </c>
+      <c r="F28" s="6" t="s">
+        <v>130</v>
+      </c>
+      <c r="G28" s="7" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="29" spans="1:7" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A29" s="5" t="s">
-        <v>104</v>
-      </c>
-      <c r="B29" s="5" t="s">
-        <v>101</v>
-      </c>
-      <c r="C29" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="D29" s="6" t="s">
-        <v>105</v>
-      </c>
-      <c r="E29" s="6" t="s">
-        <v>106</v>
-      </c>
-      <c r="F29" s="6"/>
-      <c r="G29" s="7"/>
+      <c r="A29" s="4" t="s">
+        <v>131</v>
+      </c>
+      <c r="B29" s="4" t="s">
+        <v>127</v>
+      </c>
+      <c r="C29" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="D29" s="5" t="s">
+        <v>132</v>
+      </c>
+      <c r="E29" s="5" t="s">
+        <v>133</v>
+      </c>
+      <c r="F29" s="8" t="s">
+        <v>134</v>
+      </c>
+      <c r="G29" s="9" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A30" s="2" t="s">
-        <v>107</v>
+        <v>135</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>108</v>
+        <v>136</v>
       </c>
       <c r="C30" s="2" t="s">
         <v>9</v>
       </c>
       <c r="D30" s="3" t="s">
-        <v>109</v>
+        <v>137</v>
       </c>
       <c r="E30" s="3" t="s">
-        <v>110</v>
-      </c>
-      <c r="F30" s="3"/>
-      <c r="G30" s="4"/>
+        <v>138</v>
+      </c>
+      <c r="F30" s="6" t="s">
+        <v>139</v>
+      </c>
+      <c r="G30" s="7" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="31" spans="1:7" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A31" s="5" t="s">
-        <v>111</v>
-      </c>
-      <c r="B31" s="5" t="s">
-        <v>108</v>
-      </c>
-      <c r="C31" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="D31" s="6" t="s">
-        <v>112</v>
-      </c>
-      <c r="E31" s="6" t="s">
-        <v>113</v>
-      </c>
-      <c r="F31" s="6"/>
-      <c r="G31" s="7"/>
+      <c r="A31" s="4" t="s">
+        <v>140</v>
+      </c>
+      <c r="B31" s="4" t="s">
+        <v>136</v>
+      </c>
+      <c r="C31" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="D31" s="5" t="s">
+        <v>141</v>
+      </c>
+      <c r="E31" s="5" t="s">
+        <v>142</v>
+      </c>
+      <c r="F31" s="8" t="s">
+        <v>143</v>
+      </c>
+      <c r="G31" s="9" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A32" s="2" t="s">
-        <v>114</v>
+        <v>144</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>115</v>
+        <v>145</v>
       </c>
       <c r="C32" s="2" t="s">
         <v>9</v>
       </c>
       <c r="D32" s="3" t="s">
-        <v>116</v>
+        <v>146</v>
       </c>
       <c r="E32" s="3" t="s">
-        <v>117</v>
-      </c>
-      <c r="F32" s="3"/>
-      <c r="G32" s="4"/>
+        <v>147</v>
+      </c>
+      <c r="F32" s="6" t="s">
+        <v>148</v>
+      </c>
+      <c r="G32" s="7" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="33" spans="1:7" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A33" s="5" t="s">
-        <v>118</v>
-      </c>
-      <c r="B33" s="5" t="s">
-        <v>115</v>
-      </c>
-      <c r="C33" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="D33" s="6" t="s">
-        <v>119</v>
-      </c>
-      <c r="E33" s="6" t="s">
-        <v>120</v>
-      </c>
-      <c r="F33" s="6"/>
-      <c r="G33" s="7"/>
+      <c r="A33" s="4" t="s">
+        <v>149</v>
+      </c>
+      <c r="B33" s="4" t="s">
+        <v>145</v>
+      </c>
+      <c r="C33" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="D33" s="5" t="s">
+        <v>150</v>
+      </c>
+      <c r="E33" s="5" t="s">
+        <v>151</v>
+      </c>
+      <c r="F33" s="8" t="s">
+        <v>152</v>
+      </c>
+      <c r="G33" s="9" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A34" s="2" t="s">
-        <v>121</v>
+        <v>153</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>122</v>
+        <v>154</v>
       </c>
       <c r="C34" s="2" t="s">
         <v>9</v>
       </c>
       <c r="D34" s="3" t="s">
-        <v>123</v>
+        <v>155</v>
       </c>
       <c r="E34" s="3" t="s">
-        <v>124</v>
-      </c>
-      <c r="F34" s="3"/>
-      <c r="G34" s="4"/>
+        <v>156</v>
+      </c>
+      <c r="F34" s="6" t="s">
+        <v>157</v>
+      </c>
+      <c r="G34" s="7" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="35" spans="1:7" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A35" s="5" t="s">
-        <v>125</v>
-      </c>
-      <c r="B35" s="5" t="s">
-        <v>122</v>
-      </c>
-      <c r="C35" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="D35" s="6" t="s">
-        <v>126</v>
-      </c>
-      <c r="E35" s="6" t="s">
-        <v>127</v>
-      </c>
-      <c r="F35" s="6"/>
-      <c r="G35" s="7"/>
+      <c r="A35" s="4" t="s">
+        <v>158</v>
+      </c>
+      <c r="B35" s="4" t="s">
+        <v>154</v>
+      </c>
+      <c r="C35" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D35" s="5" t="s">
+        <v>159</v>
+      </c>
+      <c r="E35" s="5" t="s">
+        <v>160</v>
+      </c>
+      <c r="F35" s="8" t="s">
+        <v>161</v>
+      </c>
+      <c r="G35" s="9" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A36" s="2" t="s">
-        <v>128</v>
+        <v>162</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>129</v>
+        <v>163</v>
       </c>
       <c r="C36" s="2" t="s">
         <v>9</v>
       </c>
       <c r="D36" s="3" t="s">
-        <v>130</v>
+        <v>164</v>
       </c>
       <c r="E36" s="3" t="s">
-        <v>131</v>
-      </c>
-      <c r="F36" s="3"/>
-      <c r="G36" s="4"/>
+        <v>165</v>
+      </c>
+      <c r="F36" s="6" t="s">
+        <v>166</v>
+      </c>
+      <c r="G36" s="7" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="37" spans="1:7" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A37" s="5" t="s">
-        <v>132</v>
-      </c>
-      <c r="B37" s="5" t="s">
-        <v>129</v>
-      </c>
-      <c r="C37" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="D37" s="6" t="s">
-        <v>133</v>
-      </c>
-      <c r="E37" s="6" t="s">
-        <v>134</v>
-      </c>
-      <c r="F37" s="6"/>
-      <c r="G37" s="7"/>
+      <c r="A37" s="4" t="s">
+        <v>167</v>
+      </c>
+      <c r="B37" s="4" t="s">
+        <v>163</v>
+      </c>
+      <c r="C37" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="D37" s="5" t="s">
+        <v>168</v>
+      </c>
+      <c r="E37" s="5" t="s">
+        <v>169</v>
+      </c>
+      <c r="F37" s="8" t="s">
+        <v>170</v>
+      </c>
+      <c r="G37" s="9" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A38" s="2" t="s">
-        <v>135</v>
+        <v>171</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>136</v>
+        <v>172</v>
       </c>
       <c r="C38" s="2" t="s">
         <v>9</v>
       </c>
       <c r="D38" s="3" t="s">
-        <v>137</v>
+        <v>173</v>
       </c>
       <c r="E38" s="3" t="s">
-        <v>138</v>
-      </c>
-      <c r="F38" s="3"/>
-      <c r="G38" s="4"/>
+        <v>174</v>
+      </c>
+      <c r="F38" s="6" t="s">
+        <v>175</v>
+      </c>
+      <c r="G38" s="7" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="39" spans="1:7" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A39" s="5" t="s">
-        <v>139</v>
-      </c>
-      <c r="B39" s="5" t="s">
-        <v>136</v>
-      </c>
-      <c r="C39" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="D39" s="6" t="s">
-        <v>140</v>
-      </c>
-      <c r="E39" s="6" t="s">
-        <v>141</v>
-      </c>
-      <c r="F39" s="6"/>
-      <c r="G39" s="7"/>
+      <c r="A39" s="4" t="s">
+        <v>176</v>
+      </c>
+      <c r="B39" s="4" t="s">
+        <v>172</v>
+      </c>
+      <c r="C39" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="D39" s="5" t="s">
+        <v>177</v>
+      </c>
+      <c r="E39" s="5" t="s">
+        <v>178</v>
+      </c>
+      <c r="F39" s="8" t="s">
+        <v>179</v>
+      </c>
+      <c r="G39" s="9" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A40" s="2" t="s">
-        <v>142</v>
+        <v>180</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>143</v>
+        <v>181</v>
       </c>
       <c r="C40" s="2" t="s">
         <v>9</v>
       </c>
       <c r="D40" s="3" t="s">
-        <v>144</v>
+        <v>182</v>
       </c>
       <c r="E40" s="3" t="s">
-        <v>145</v>
-      </c>
-      <c r="F40" s="3"/>
-      <c r="G40" s="4"/>
+        <v>183</v>
+      </c>
+      <c r="F40" s="6" t="s">
+        <v>184</v>
+      </c>
+      <c r="G40" s="7" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="41" spans="1:7" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A41" s="5" t="s">
-        <v>146</v>
-      </c>
-      <c r="B41" s="5" t="s">
-        <v>143</v>
-      </c>
-      <c r="C41" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="D41" s="6" t="s">
-        <v>147</v>
-      </c>
-      <c r="E41" s="6" t="s">
-        <v>148</v>
-      </c>
-      <c r="F41" s="6"/>
-      <c r="G41" s="7"/>
+      <c r="A41" s="4" t="s">
+        <v>185</v>
+      </c>
+      <c r="B41" s="4" t="s">
+        <v>181</v>
+      </c>
+      <c r="C41" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D41" s="5" t="s">
+        <v>186</v>
+      </c>
+      <c r="E41" s="5" t="s">
+        <v>187</v>
+      </c>
+      <c r="F41" s="8" t="s">
+        <v>188</v>
+      </c>
+      <c r="G41" s="9" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A42" s="2" t="s">
-        <v>149</v>
+        <v>189</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>150</v>
+        <v>190</v>
       </c>
       <c r="C42" s="2" t="s">
         <v>9</v>
       </c>
       <c r="D42" s="3" t="s">
-        <v>151</v>
+        <v>191</v>
       </c>
       <c r="E42" s="3" t="s">
-        <v>152</v>
-      </c>
-      <c r="F42" s="3"/>
-      <c r="G42" s="4"/>
+        <v>192</v>
+      </c>
+      <c r="F42" s="6" t="s">
+        <v>193</v>
+      </c>
+      <c r="G42" s="7" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="43" spans="1:7" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A43" s="5" t="s">
-        <v>153</v>
-      </c>
-      <c r="B43" s="5" t="s">
-        <v>150</v>
-      </c>
-      <c r="C43" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="D43" s="6" t="s">
-        <v>154</v>
-      </c>
-      <c r="E43" s="6" t="s">
-        <v>155</v>
-      </c>
-      <c r="F43" s="6"/>
-      <c r="G43" s="7"/>
+      <c r="A43" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="B43" s="4" t="s">
+        <v>190</v>
+      </c>
+      <c r="C43" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D43" s="5" t="s">
+        <v>195</v>
+      </c>
+      <c r="E43" s="5" t="s">
+        <v>196</v>
+      </c>
+      <c r="F43" s="8" t="s">
+        <v>197</v>
+      </c>
+      <c r="G43" s="9" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A44" s="2" t="s">
-        <v>156</v>
+        <v>198</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>157</v>
+        <v>199</v>
       </c>
       <c r="C44" s="2" t="s">
         <v>9</v>
       </c>
       <c r="D44" s="3" t="s">
-        <v>158</v>
+        <v>200</v>
       </c>
       <c r="E44" s="3" t="s">
-        <v>159</v>
-      </c>
-      <c r="F44" s="3"/>
-      <c r="G44" s="4"/>
+        <v>201</v>
+      </c>
+      <c r="F44" s="6" t="s">
+        <v>202</v>
+      </c>
+      <c r="G44" s="7" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="45" spans="1:7" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A45" s="5" t="s">
-        <v>160</v>
-      </c>
-      <c r="B45" s="5" t="s">
-        <v>157</v>
-      </c>
-      <c r="C45" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="D45" s="6" t="s">
-        <v>161</v>
-      </c>
-      <c r="E45" s="6" t="s">
-        <v>162</v>
-      </c>
-      <c r="F45" s="6"/>
-      <c r="G45" s="7"/>
+      <c r="A45" s="4" t="s">
+        <v>203</v>
+      </c>
+      <c r="B45" s="4" t="s">
+        <v>199</v>
+      </c>
+      <c r="C45" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="D45" s="5" t="s">
+        <v>204</v>
+      </c>
+      <c r="E45" s="5" t="s">
+        <v>205</v>
+      </c>
+      <c r="F45" s="8" t="s">
+        <v>206</v>
+      </c>
+      <c r="G45" s="9" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A46" s="2" t="s">
-        <v>163</v>
+        <v>207</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>164</v>
+        <v>208</v>
       </c>
       <c r="C46" s="2" t="s">
         <v>9</v>
       </c>
       <c r="D46" s="3" t="s">
-        <v>165</v>
+        <v>209</v>
       </c>
       <c r="E46" s="3" t="s">
-        <v>166</v>
-      </c>
-      <c r="F46" s="3"/>
-      <c r="G46" s="4"/>
+        <v>210</v>
+      </c>
+      <c r="F46" s="6" t="s">
+        <v>211</v>
+      </c>
+      <c r="G46" s="7" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="47" spans="1:7" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A47" s="5" t="s">
-        <v>167</v>
-      </c>
-      <c r="B47" s="5" t="s">
-        <v>164</v>
-      </c>
-      <c r="C47" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="D47" s="6" t="s">
-        <v>168</v>
-      </c>
-      <c r="E47" s="6" t="s">
-        <v>169</v>
-      </c>
-      <c r="F47" s="6"/>
-      <c r="G47" s="7"/>
+      <c r="A47" s="4" t="s">
+        <v>212</v>
+      </c>
+      <c r="B47" s="4" t="s">
+        <v>208</v>
+      </c>
+      <c r="C47" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D47" s="5" t="s">
+        <v>213</v>
+      </c>
+      <c r="E47" s="5" t="s">
+        <v>214</v>
+      </c>
+      <c r="F47" s="8" t="s">
+        <v>215</v>
+      </c>
+      <c r="G47" s="9" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A48" s="2" t="s">
-        <v>170</v>
+        <v>216</v>
       </c>
       <c r="B48" s="2" t="s">
-        <v>171</v>
+        <v>217</v>
       </c>
       <c r="C48" s="2" t="s">
         <v>9</v>
       </c>
       <c r="D48" s="3" t="s">
-        <v>172</v>
+        <v>218</v>
       </c>
       <c r="E48" s="3" t="s">
-        <v>75</v>
-      </c>
-      <c r="F48" s="3"/>
-      <c r="G48" s="4"/>
+        <v>93</v>
+      </c>
+      <c r="F48" s="6" t="s">
+        <v>219</v>
+      </c>
+      <c r="G48" s="7" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="49" spans="1:7" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A49" s="5" t="s">
-        <v>173</v>
-      </c>
-      <c r="B49" s="5" t="s">
-        <v>171</v>
-      </c>
-      <c r="C49" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="D49" s="6" t="s">
-        <v>174</v>
-      </c>
-      <c r="E49" s="6" t="s">
-        <v>175</v>
-      </c>
-      <c r="F49" s="6"/>
-      <c r="G49" s="7"/>
+      <c r="A49" s="4" t="s">
+        <v>220</v>
+      </c>
+      <c r="B49" s="4" t="s">
+        <v>217</v>
+      </c>
+      <c r="C49" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="D49" s="5" t="s">
+        <v>221</v>
+      </c>
+      <c r="E49" s="5" t="s">
+        <v>222</v>
+      </c>
+      <c r="F49" s="8" t="s">
+        <v>223</v>
+      </c>
+      <c r="G49" s="9" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A50" s="2" t="s">
-        <v>176</v>
+        <v>224</v>
       </c>
       <c r="B50" s="2" t="s">
-        <v>177</v>
+        <v>225</v>
       </c>
       <c r="C50" s="2" t="s">
         <v>9</v>
       </c>
       <c r="D50" s="3" t="s">
-        <v>178</v>
+        <v>226</v>
       </c>
       <c r="E50" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="F50" s="3"/>
-      <c r="G50" s="4"/>
+        <v>227</v>
+      </c>
+      <c r="F50" s="6" t="s">
+        <v>228</v>
+      </c>
+      <c r="G50" s="7" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="51" spans="1:7" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A51" s="5" t="s">
-        <v>180</v>
-      </c>
-      <c r="B51" s="5" t="s">
-        <v>177</v>
-      </c>
-      <c r="C51" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="D51" s="6" t="s">
-        <v>181</v>
-      </c>
-      <c r="E51" s="6" t="s">
-        <v>182</v>
-      </c>
-      <c r="F51" s="6"/>
-      <c r="G51" s="7"/>
+      <c r="A51" s="4" t="s">
+        <v>229</v>
+      </c>
+      <c r="B51" s="4" t="s">
+        <v>225</v>
+      </c>
+      <c r="C51" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="D51" s="5" t="s">
+        <v>230</v>
+      </c>
+      <c r="E51" s="5" t="s">
+        <v>231</v>
+      </c>
+      <c r="F51" s="8" t="s">
+        <v>232</v>
+      </c>
+      <c r="G51" s="9" t="s">
+        <v>13</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>